<commit_message>
Refactor pool management components to include salt system handling
- Updated pool-related forms and data structures to incorporate a new hasSaltSystem field, enhancing the ability to manage pools with salt systems.
- Modified the ModalAddPool and ModalEditPool components to handle salt system selection and update pool types accordingly.
- Adjusted CSV and Excel import templates to reflect the new hasSaltSystem field, ensuring consistency in data handling.
- Enhanced maintenance records management to differentiate between filter and salt system maintenance, improving user experience and data clarity.
- Updated various components to streamline the integration of salt system features, including UI adjustments and validation logic.
</commit_message>
<xml_diff>
--- a/public/templates/client_import_template.xlsx
+++ b/public/templates/client_import_template.xlsx
@@ -452,7 +452,7 @@
         <v>poolNotes</v>
       </c>
       <c r="R1" t="str">
-        <v>poolType</v>
+        <v>hasSaltSystem</v>
       </c>
       <c r="S1" t="str">
         <v>poolState</v>
@@ -526,7 +526,7 @@
         <v>notes</v>
       </c>
       <c r="R2" t="str">
-        <v>Chlorine</v>
+        <v>FALSE (Type TRUE or FALSE)</v>
       </c>
       <c r="S2" t="str">
         <v>FL</v>

</xml_diff>